<commit_message>
feat: creation tables et insertion donnees sources
</commit_message>
<xml_diff>
--- a/sources/referentiel.xlsx
+++ b/sources/referentiel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Boly-\Desktop\WaveOps\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40C11333-557F-4BA6-AD96-9EF4612A1D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBE6CD1-F80B-4AEB-8964-F61B7F3B109A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{663ACB3C-F968-4EE1-B0D7-126396464402}"/>
   </bookViews>
@@ -38,10 +38,134 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+  <si>
+    <t>agence</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>responsable</t>
+  </si>
+  <si>
+    <t>segment</t>
+  </si>
+  <si>
+    <t>Paris Centre</t>
+  </si>
+  <si>
+    <t>Ile-de-France</t>
+  </si>
+  <si>
+    <t>Marie Dubois</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Paris Nord</t>
+  </si>
+  <si>
+    <t>Jean Martin</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Lyon Part-Dieu</t>
+  </si>
+  <si>
+    <t>Auvergne-Rhone-Alpes</t>
+  </si>
+  <si>
+    <t>Sophie Bernard</t>
+  </si>
+  <si>
+    <t>Pro</t>
+  </si>
+  <si>
+    <t>Marseille Vieux-Port</t>
+  </si>
+  <si>
+    <t>PACA</t>
+  </si>
+  <si>
+    <t>Pierre Petit</t>
+  </si>
+  <si>
+    <t>Bordeaux Centre</t>
+  </si>
+  <si>
+    <t>Nouvelle-Aquitaine</t>
+  </si>
+  <si>
+    <t>Claire Moreau</t>
+  </si>
+  <si>
+    <t>Jeune</t>
+  </si>
+  <si>
+    <t>Lille Grand Place</t>
+  </si>
+  <si>
+    <t>Hauts-de-France</t>
+  </si>
+  <si>
+    <t>Thomas Leroy</t>
+  </si>
+  <si>
+    <t>Nantes Centre</t>
+  </si>
+  <si>
+    <t>Pays de la Loire</t>
+  </si>
+  <si>
+    <t>Emma Roux</t>
+  </si>
+  <si>
+    <t>Strasbourg Centre</t>
+  </si>
+  <si>
+    <t>Grand Est</t>
+  </si>
+  <si>
+    <t>Nicolas Simon</t>
+  </si>
+  <si>
+    <t>Toulouse Wilson</t>
+  </si>
+  <si>
+    <t>Occitanie</t>
+  </si>
+  <si>
+    <t>Julie Laurent</t>
+  </si>
+  <si>
+    <t>Rennes Centre</t>
+  </si>
+  <si>
+    <t>Bretagne</t>
+  </si>
+  <si>
+    <t>Marc Dupont</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -69,13 +193,54 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -86,6 +251,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{799313C7-89C6-4AA8-9CD4-4C51E4F6D57A}" name="Tableau1" displayName="Tableau1" ref="A1:D11" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:D11" xr:uid="{799313C7-89C6-4AA8-9CD4-4C51E4F6D57A}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{82FCA12F-8C85-48AF-948F-E0B961D474D7}" name="agence" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{E90C9B56-24D8-4808-A31C-47E9A44AEF30}" name="region" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{6445F4DB-B9B9-468B-9DB0-BEF2F2F5A70F}" name="responsable" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{974C19FA-095F-471A-800A-C86B25DDB2C5}" name="segment" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,9 +583,172 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14601BD4-4CA9-4A42-9C45-B4AA99A11E20}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>